<commit_message>
LITE-35404 Release 1.0.4: bring the 1.0.4.RC content onto master
master carried only the Google Workspace audit report from CG-762. Everything
newer lives on tag 1.0.4.RC, which is on no branch: the Google Workspace
Billing report, the Consumption column on the audit report, and the shared
reports/http.py. Olivetti needs this code in their Connect account and should
not be pointed at a release candidate.

The two lines have unrelated git histories, with separate root commits, so
there is nothing to merge. This sets the tree to 1.0.4.RC, with four changes:

- .idea/ is left out, it is already in .gitignore
- tests/__init__.py keeps the CloudBlue copyright line from master
- pyproject.toml version 1.0.1 -> 1.0.4 and reports.json version 1.0 -> 1.0.4,
  both of which had fallen behind the tags
- CHANGELOG entry for 1.0.4

Tag 1.0.4.RC still points at the original commits.
</commit_message>
<xml_diff>
--- a/reports/google_workspace_report/templates/xlsx/template.xlsx
+++ b/reports/google_workspace_report/templates/xlsx/template.xlsx
@@ -1,30 +1,30 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27628"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10112"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\filip.djordjevic\source\repos\google-workspace-connect-report\reports\google_workspace_report\templates\xlsx\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/dfranco00/Sites/google-workspace-connect-report/reports/google_workspace_report/templates/xlsx/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{71760C4C-F3FD-4A9E-BBFA-3A3BB3CAA1EB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E35C4D3B-36EF-284E-9270-5F343FC2D79F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2652" yWindow="2652" windowWidth="17280" windowHeight="8964" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="500" windowWidth="35840" windowHeight="19380" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Data" sheetId="1" r:id="rId1"/>
     <sheet name="Info" sheetId="2" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Data!$A$1:$AZ$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Data!$A$1:$BA$1</definedName>
   </definedNames>
   <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="69" uniqueCount="69">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="70" uniqueCount="70">
   <si>
     <t>Subscription ID</t>
   </si>
@@ -271,6 +271,9 @@
   </si>
   <si>
     <t>Error Details</t>
+  </si>
+  <si>
+    <t>Consumption</t>
   </si>
 </sst>
 </file>
@@ -648,42 +651,42 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:AZ15"/>
-  <sheetFormatPr defaultColWidth="8.77734375" defaultRowHeight="14.4" outlineLevelCol="1" x14ac:dyDescent="0.3"/>
+  <dimension ref="A1:BA15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" outlineLevelCol="1" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="26.33203125" style="3" customWidth="1" outlineLevel="1"/>
-    <col min="2" max="19" width="20" style="3" customWidth="1"/>
-    <col min="20" max="23" width="18.77734375" style="4" customWidth="1" outlineLevel="1"/>
-    <col min="24" max="25" width="25" style="4" customWidth="1" outlineLevel="1"/>
-    <col min="26" max="29" width="18.77734375" style="3" customWidth="1"/>
-    <col min="30" max="30" width="17.21875" style="3" customWidth="1"/>
-    <col min="31" max="31" width="20" style="3" customWidth="1" outlineLevel="1"/>
-    <col min="32" max="32" width="17.77734375" style="3" customWidth="1"/>
-    <col min="33" max="33" width="17.77734375" style="3" customWidth="1" outlineLevel="1"/>
-    <col min="34" max="34" width="17.77734375" style="3" customWidth="1"/>
-    <col min="35" max="35" width="19.33203125" style="3" customWidth="1" outlineLevel="1"/>
-    <col min="36" max="36" width="45.77734375" style="3" customWidth="1" outlineLevel="1"/>
-    <col min="37" max="37" width="20" style="3" customWidth="1"/>
-    <col min="38" max="38" width="19.33203125" style="3" customWidth="1" outlineLevel="1"/>
-    <col min="39" max="39" width="45.77734375" style="3" customWidth="1" outlineLevel="1"/>
-    <col min="40" max="40" width="20" style="3" customWidth="1"/>
-    <col min="41" max="41" width="19.33203125" style="3" customWidth="1" outlineLevel="1"/>
-    <col min="42" max="42" width="45.77734375" style="3" customWidth="1" outlineLevel="1"/>
-    <col min="43" max="43" width="20" style="3" customWidth="1"/>
-    <col min="44" max="44" width="20" style="3" customWidth="1" outlineLevel="1"/>
-    <col min="45" max="45" width="45.77734375" style="3" customWidth="1"/>
-    <col min="46" max="46" width="15" style="3" customWidth="1" outlineLevel="1"/>
-    <col min="47" max="47" width="45.77734375" style="3" customWidth="1"/>
-    <col min="48" max="48" width="20" style="3" customWidth="1" outlineLevel="1"/>
-    <col min="49" max="49" width="45.77734375" style="3" customWidth="1"/>
-    <col min="50" max="50" width="15" style="3" customWidth="1" outlineLevel="1"/>
-    <col min="51" max="51" width="45.77734375" style="3" customWidth="1"/>
-    <col min="52" max="52" width="18.6640625" style="3" customWidth="1"/>
-    <col min="53" max="53" width="8.77734375" style="3" customWidth="1"/>
-    <col min="54" max="16384" width="8.77734375" style="3"/>
+    <col min="2" max="20" width="20" style="3" customWidth="1"/>
+    <col min="21" max="24" width="18.83203125" style="4" customWidth="1" outlineLevel="1"/>
+    <col min="25" max="26" width="25" style="4" customWidth="1" outlineLevel="1"/>
+    <col min="27" max="30" width="18.83203125" style="3" customWidth="1"/>
+    <col min="31" max="31" width="17.1640625" style="3" customWidth="1"/>
+    <col min="32" max="32" width="20" style="3" customWidth="1" outlineLevel="1"/>
+    <col min="33" max="33" width="17.83203125" style="3" customWidth="1"/>
+    <col min="34" max="34" width="17.83203125" style="3" customWidth="1" outlineLevel="1"/>
+    <col min="35" max="35" width="17.83203125" style="3" customWidth="1"/>
+    <col min="36" max="36" width="19.33203125" style="3" customWidth="1" outlineLevel="1"/>
+    <col min="37" max="37" width="45.83203125" style="3" customWidth="1" outlineLevel="1"/>
+    <col min="38" max="38" width="20" style="3" customWidth="1"/>
+    <col min="39" max="39" width="19.33203125" style="3" customWidth="1" outlineLevel="1"/>
+    <col min="40" max="40" width="45.83203125" style="3" customWidth="1" outlineLevel="1"/>
+    <col min="41" max="41" width="20" style="3" customWidth="1"/>
+    <col min="42" max="42" width="19.33203125" style="3" customWidth="1" outlineLevel="1"/>
+    <col min="43" max="43" width="45.83203125" style="3" customWidth="1" outlineLevel="1"/>
+    <col min="44" max="44" width="20" style="3" customWidth="1"/>
+    <col min="45" max="45" width="20" style="3" customWidth="1" outlineLevel="1"/>
+    <col min="46" max="46" width="45.83203125" style="3" customWidth="1"/>
+    <col min="47" max="47" width="15" style="3" customWidth="1" outlineLevel="1"/>
+    <col min="48" max="48" width="45.83203125" style="3" customWidth="1"/>
+    <col min="49" max="49" width="20" style="3" customWidth="1" outlineLevel="1"/>
+    <col min="50" max="50" width="45.83203125" style="3" customWidth="1"/>
+    <col min="51" max="51" width="15" style="3" customWidth="1" outlineLevel="1"/>
+    <col min="52" max="52" width="45.83203125" style="3" customWidth="1"/>
+    <col min="53" max="53" width="18.6640625" style="3" customWidth="1"/>
+    <col min="54" max="54" width="8.83203125" style="3" customWidth="1"/>
+    <col min="55" max="16384" width="8.83203125" style="3"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:52" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:53" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -727,234 +730,236 @@
         <v>53</v>
       </c>
       <c r="O1" s="1" t="s">
+        <v>69</v>
+      </c>
+      <c r="P1" s="1" t="s">
         <v>61</v>
       </c>
-      <c r="P1" s="1" t="s">
+      <c r="Q1" s="1" t="s">
         <v>59</v>
       </c>
-      <c r="Q1" s="1" t="s">
+      <c r="R1" s="1" t="s">
         <v>60</v>
       </c>
-      <c r="R1" s="1" t="s">
+      <c r="S1" s="1" t="s">
         <v>64</v>
       </c>
-      <c r="S1" s="1" t="s">
+      <c r="T1" s="1" t="s">
         <v>63</v>
       </c>
-      <c r="T1" s="2" t="s">
+      <c r="U1" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="U1" s="2" t="s">
+      <c r="V1" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="V1" s="2" t="s">
+      <c r="W1" s="2" t="s">
         <v>55</v>
       </c>
-      <c r="W1" s="2" t="s">
+      <c r="X1" s="2" t="s">
         <v>56</v>
       </c>
-      <c r="X1" s="2" t="s">
+      <c r="Y1" s="2" t="s">
         <v>57</v>
       </c>
-      <c r="Y1" s="2" t="s">
+      <c r="Z1" s="2" t="s">
         <v>58</v>
       </c>
-      <c r="Z1" s="1" t="s">
+      <c r="AA1" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="AA1" s="1" t="s">
+      <c r="AB1" s="1" t="s">
         <v>52</v>
       </c>
-      <c r="AB1" s="1" t="s">
+      <c r="AC1" s="1" t="s">
         <v>66</v>
       </c>
-      <c r="AC1" s="1" t="s">
+      <c r="AD1" s="1" t="s">
         <v>67</v>
       </c>
-      <c r="AD1" s="1" t="s">
+      <c r="AE1" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="AE1" s="1" t="s">
+      <c r="AF1" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="AF1" s="1" t="s">
+      <c r="AG1" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="AG1" s="1" t="s">
+      <c r="AH1" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="AH1" s="1" t="s">
+      <c r="AI1" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="AI1" s="1" t="s">
+      <c r="AJ1" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="AJ1" s="1" t="s">
+      <c r="AK1" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="AK1" s="1" t="s">
+      <c r="AL1" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="AL1" s="1" t="s">
+      <c r="AM1" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="AM1" s="1" t="s">
+      <c r="AN1" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="AN1" s="1" t="s">
+      <c r="AO1" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="AO1" s="1" t="s">
+      <c r="AP1" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="AP1" s="1" t="s">
+      <c r="AQ1" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="AQ1" s="1" t="s">
+      <c r="AR1" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="AR1" s="1" t="s">
+      <c r="AS1" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="AS1" s="1" t="s">
+      <c r="AT1" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="AT1" s="1" t="s">
+      <c r="AU1" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="AU1" s="1" t="s">
+      <c r="AV1" s="1" t="s">
         <v>29</v>
       </c>
-      <c r="AV1" s="1" t="s">
+      <c r="AW1" s="1" t="s">
         <v>30</v>
       </c>
-      <c r="AW1" s="1" t="s">
+      <c r="AX1" s="1" t="s">
         <v>31</v>
       </c>
-      <c r="AX1" s="1" t="s">
+      <c r="AY1" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="AY1" s="1" t="s">
+      <c r="AZ1" s="1" t="s">
         <v>33</v>
       </c>
-      <c r="AZ1" s="1" t="s">
+      <c r="BA1" s="1" t="s">
         <v>68</v>
       </c>
     </row>
-    <row r="2" spans="1:52" x14ac:dyDescent="0.3">
-      <c r="T2" s="5"/>
+    <row r="2" spans="1:53" x14ac:dyDescent="0.2">
       <c r="U2" s="5"/>
       <c r="V2" s="5"/>
       <c r="W2" s="5"/>
       <c r="X2" s="5"/>
       <c r="Y2" s="5"/>
-    </row>
-    <row r="3" spans="1:52" x14ac:dyDescent="0.3">
-      <c r="T3" s="5"/>
+      <c r="Z2" s="5"/>
+    </row>
+    <row r="3" spans="1:53" x14ac:dyDescent="0.2">
       <c r="U3" s="5"/>
       <c r="V3" s="5"/>
       <c r="W3" s="5"/>
       <c r="X3" s="5"/>
       <c r="Y3" s="5"/>
-    </row>
-    <row r="4" spans="1:52" x14ac:dyDescent="0.3">
-      <c r="T4" s="5"/>
+      <c r="Z3" s="5"/>
+    </row>
+    <row r="4" spans="1:53" x14ac:dyDescent="0.2">
       <c r="U4" s="5"/>
       <c r="V4" s="5"/>
       <c r="W4" s="5"/>
       <c r="X4" s="5"/>
       <c r="Y4" s="5"/>
-    </row>
-    <row r="5" spans="1:52" x14ac:dyDescent="0.3">
-      <c r="T5" s="5"/>
+      <c r="Z4" s="5"/>
+    </row>
+    <row r="5" spans="1:53" x14ac:dyDescent="0.2">
       <c r="U5" s="5"/>
       <c r="V5" s="5"/>
       <c r="W5" s="5"/>
       <c r="X5" s="5"/>
       <c r="Y5" s="5"/>
-    </row>
-    <row r="6" spans="1:52" x14ac:dyDescent="0.3">
-      <c r="T6" s="5"/>
+      <c r="Z5" s="5"/>
+    </row>
+    <row r="6" spans="1:53" x14ac:dyDescent="0.2">
       <c r="U6" s="5"/>
       <c r="V6" s="5"/>
       <c r="W6" s="5"/>
       <c r="X6" s="5"/>
       <c r="Y6" s="5"/>
-    </row>
-    <row r="7" spans="1:52" x14ac:dyDescent="0.3">
-      <c r="T7" s="5"/>
+      <c r="Z6" s="5"/>
+    </row>
+    <row r="7" spans="1:53" x14ac:dyDescent="0.2">
       <c r="U7" s="5"/>
       <c r="V7" s="5"/>
       <c r="W7" s="5"/>
       <c r="X7" s="5"/>
       <c r="Y7" s="5"/>
-    </row>
-    <row r="8" spans="1:52" x14ac:dyDescent="0.3">
-      <c r="T8" s="5"/>
+      <c r="Z7" s="5"/>
+    </row>
+    <row r="8" spans="1:53" x14ac:dyDescent="0.2">
       <c r="U8" s="5"/>
       <c r="V8" s="5"/>
       <c r="W8" s="5"/>
       <c r="X8" s="5"/>
       <c r="Y8" s="5"/>
-    </row>
-    <row r="9" spans="1:52" x14ac:dyDescent="0.3">
-      <c r="T9" s="5"/>
+      <c r="Z8" s="5"/>
+    </row>
+    <row r="9" spans="1:53" x14ac:dyDescent="0.2">
       <c r="U9" s="5"/>
       <c r="V9" s="5"/>
       <c r="W9" s="5"/>
       <c r="X9" s="5"/>
       <c r="Y9" s="5"/>
-    </row>
-    <row r="10" spans="1:52" x14ac:dyDescent="0.3">
-      <c r="T10" s="5"/>
+      <c r="Z9" s="5"/>
+    </row>
+    <row r="10" spans="1:53" x14ac:dyDescent="0.2">
       <c r="U10" s="5"/>
       <c r="V10" s="5"/>
       <c r="W10" s="5"/>
       <c r="X10" s="5"/>
       <c r="Y10" s="5"/>
-    </row>
-    <row r="11" spans="1:52" x14ac:dyDescent="0.3">
-      <c r="T11" s="5"/>
+      <c r="Z10" s="5"/>
+    </row>
+    <row r="11" spans="1:53" x14ac:dyDescent="0.2">
       <c r="U11" s="5"/>
       <c r="V11" s="5"/>
       <c r="W11" s="5"/>
       <c r="X11" s="5"/>
       <c r="Y11" s="5"/>
-    </row>
-    <row r="12" spans="1:52" x14ac:dyDescent="0.3">
-      <c r="T12" s="5"/>
+      <c r="Z11" s="5"/>
+    </row>
+    <row r="12" spans="1:53" x14ac:dyDescent="0.2">
       <c r="U12" s="5"/>
       <c r="V12" s="5"/>
       <c r="W12" s="5"/>
       <c r="X12" s="5"/>
       <c r="Y12" s="5"/>
-    </row>
-    <row r="13" spans="1:52" x14ac:dyDescent="0.3">
-      <c r="T13" s="5"/>
+      <c r="Z12" s="5"/>
+    </row>
+    <row r="13" spans="1:53" x14ac:dyDescent="0.2">
       <c r="U13" s="5"/>
       <c r="V13" s="5"/>
       <c r="W13" s="5"/>
       <c r="X13" s="5"/>
       <c r="Y13" s="5"/>
-    </row>
-    <row r="14" spans="1:52" x14ac:dyDescent="0.3">
-      <c r="T14" s="5"/>
+      <c r="Z13" s="5"/>
+    </row>
+    <row r="14" spans="1:53" x14ac:dyDescent="0.2">
       <c r="U14" s="5"/>
       <c r="V14" s="5"/>
       <c r="W14" s="5"/>
       <c r="X14" s="5"/>
       <c r="Y14" s="5"/>
-    </row>
-    <row r="15" spans="1:52" x14ac:dyDescent="0.3">
-      <c r="T15" s="5"/>
+      <c r="Z14" s="5"/>
+    </row>
+    <row r="15" spans="1:53" x14ac:dyDescent="0.2">
       <c r="U15" s="5"/>
       <c r="V15" s="5"/>
       <c r="W15" s="5"/>
       <c r="X15" s="5"/>
       <c r="Y15" s="5"/>
+      <c r="Z15" s="5"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:AZ1" xr:uid="{00000000-0001-0000-0000-000000000000}"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -962,19 +967,19 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:B9"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="50" customWidth="1"/>
     <col min="2" max="2" width="180" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" ht="31.2" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:2" ht="31" x14ac:dyDescent="0.2">
       <c r="A1" s="8" t="s">
         <v>36</v>
       </c>
       <c r="B1" s="9"/>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A2" s="6" t="s">
         <v>37</v>
       </c>
@@ -982,7 +987,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A3" s="6" t="s">
         <v>39</v>
       </c>
@@ -990,7 +995,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A4" s="6" t="s">
         <v>41</v>
       </c>
@@ -998,7 +1003,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A5" s="6" t="s">
         <v>42</v>
       </c>
@@ -1006,7 +1011,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A6" s="6" t="s">
         <v>43</v>
       </c>
@@ -1014,7 +1019,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A7" s="6" t="s">
         <v>45</v>
       </c>
@@ -1022,7 +1027,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A8" s="6" t="s">
         <v>47</v>
       </c>
@@ -1030,7 +1035,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="9" spans="1:2" ht="409.6" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:2" ht="409.6" x14ac:dyDescent="0.2">
       <c r="A9" s="6" t="s">
         <v>49</v>
       </c>

</xml_diff>